<commit_message>
filiais x vendas redondinho
</commit_message>
<xml_diff>
--- a/projecao_produtos_2026-03-10.xlsx
+++ b/projecao_produtos_2026-03-10.xlsx
@@ -577,7 +577,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Projeção de Estoque por Produto — Gerado em 10/03/2026 16:37</t>
+          <t>Projeção de Estoque por Produto — Gerado em 10/03/2026 17:18</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
     <row r="29" ht="22" customHeight="1">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Relatório gerado em: 10/03/2026 16:37</t>
+          <t>Relatório gerado em: 10/03/2026 17:18</t>
         </is>
       </c>
     </row>

</xml_diff>